<commit_message>
Regenerate warehouse db and Excel output
</commit_message>
<xml_diff>
--- a/output/portfolio_exception_sheet.xlsx
+++ b/output/portfolio_exception_sheet.xlsx
@@ -144,9 +144,7 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -519,8 +517,8 @@
   <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="57" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="1" max="1"/>
+    <col width="33" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
@@ -537,7 +535,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Report Date: 2026-07-21 | Source Ledgers: IBOR vs CBOR</t>
+          <t>Report Date: 2026-07-21 | Source: SQL Database Layer</t>
         </is>
       </c>
     </row>
@@ -634,7 +632,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Collins St Private Equity</t>
+          <t>Collins St Private Equity Fund</t>
         </is>
       </c>
       <c r="C7" s="6" t="n">

</xml_diff>